<commit_message>
Reprinted set after the potency and Wedding Cake passes; archives, lists and engagement report regenerated
The 172 documents reprinted as vector PDF with the potency grades from the owner's
specification and Wedding Cake's attributes; the merged tranche and by-round documents and
the four archives (HTML, vector PDF and Word of every certificate) rebuilt from them. No
page carries an embedded image; every document appears exactly once per format. The retest
and release certificate lists and the engagement report regenerated from the current data
and record.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyBhj47i7bhaCyNMB1iwdv
</commit_message>
<xml_diff>
--- a/deliverables/qc_gap_analysis/tracker/CoQ_Initial_List_2026-09-17.xlsx
+++ b/deliverables/qc_gap_analysis/tracker/CoQ_Initial_List_2026-09-17.xlsx
@@ -5841,7 +5841,11 @@
           <t>Wedding Cake</t>
         </is>
       </c>
-      <c r="I47" s="3" t="inlineStr"/>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>HYBRID · THC · MACHINE TRIMMED (TO BE DETERMINED)</t>
+        </is>
+      </c>
       <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" s="3" t="inlineStr"/>
       <c r="L47" s="3" t="inlineStr"/>
@@ -17865,7 +17869,11 @@
           <t>Wedding Cake</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>HYBRID · THC · MACHINE TRIMMED (TO BE DETERMINED)</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="3" t="inlineStr"/>
       <c r="L16" s="3" t="inlineStr"/>

</xml_diff>